<commit_message>
Update Readme and Image
</commit_message>
<xml_diff>
--- a/Credentials/position.xlsx
+++ b/Credentials/position.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="option_chain" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="143">
   <si>
     <t>expiry</t>
   </si>
@@ -449,6 +449,9 @@
   </si>
   <si>
     <t>Exit_All 12:57:39 PM</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
 </sst>
 </file>
@@ -970,6 +973,7 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2554,6 +2558,9 @@
       <c r="I10" s="3">
         <v>25450</v>
       </c>
+      <c r="J10" s="4" t="s">
+        <v>142</v>
+      </c>
       <c r="K10">
         <v>34.9</v>
       </c>
@@ -2720,6 +2727,9 @@
       </c>
       <c r="G14" s="4">
         <v>32.950000000000003</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>142</v>
       </c>
       <c r="I14" s="3">
         <v>25650</v>

</xml_diff>